<commit_message>
Subiendo imágnes de pcb y esquemático
</commit_message>
<xml_diff>
--- a/Proyecto 1C/Varios/Lista de Componentes.xlsx
+++ b/Proyecto 1C/Varios/Lista de Componentes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://frbautneduar-my.sharepoint.com/personal/dochoacruz_frba_utn_edu_ar/Documents/UTN-FRBA/Nivel 5/Electrónica de Potencia/Proyecto G2/Proyecto 1C/Varios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84877BBB-930F-42E6-911B-D9B9BC49E5CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{84877BBB-930F-42E6-911B-D9B9BC49E5CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67409924-27DB-4C61-9000-6A165777C029}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{186BFB50-1C85-497D-BC27-BC626D47804A}"/>
   </bookViews>
@@ -974,7 +974,7 @@
       <c r="I17" s="4"/>
       <c r="J17" s="4"/>
       <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
+      <c r="L17" s="9"/>
     </row>
     <row r="18" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B18" s="12">
@@ -993,7 +993,7 @@
       <c r="I18" s="4"/>
       <c r="J18" s="4"/>
       <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
+      <c r="L18" s="9"/>
     </row>
     <row r="19" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B19" s="1">

</xml_diff>